<commit_message>
feat(data): author dedicated elation damage inputs
</commit_message>
<xml_diff>
--- a/config/data/Operation.xlsx
+++ b/config/data/Operation.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operation" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Operation" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J748"/>
+  <dimension ref="A1:J749"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.7109375" customWidth="1" min="1" max="1"/>
@@ -31109,6 +31109,44 @@
       <c r="J748" t="inlineStr">
         <is>
           <t>{"type":"ModifyEffect","effect_id":1030503,"stack_delta_expression_id":1031114}</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="B749" t="n">
+        <v>970201</v>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>policy.probe.elation.operation.explicit-self-damage</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+      <c r="E749" t="n">
+        <v>24051</v>
+      </c>
+      <c r="G749" t="inlineStr">
+        <is>
+          <t>Fault</t>
+        </is>
+      </c>
+      <c r="H749" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="I749" t="inlineStr">
+        <is>
+          <t>Rollback</t>
+        </is>
+      </c>
+      <c r="J749" t="inlineStr">
+        <is>
+          <t>{"type":"ElationDamage","base_damage_expression_id":970101,"original_multiplier_expression_id":970102,"meter_multiplier_expression_id":970111,"merrymaking_expression_id":970103,"target_resistance_expression_id":970104,"penetration_expression_id":970105,"resistance_minimum_expression_id":970106,"resistance_maximum_expression_id":970107,"unbroken_multiplier_expression_id":970108,"element":"Fire","can_crit":false}</t>
         </is>
       </c>
     </row>

</xml_diff>